<commit_message>
add next order date field
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="31">
   <si>
     <t>Model</t>
   </si>
@@ -59,6 +59,9 @@
   </si>
   <si>
     <t>Next Order</t>
+  </si>
+  <si>
+    <t>Next Order Date</t>
   </si>
   <si>
     <t>Next ETA</t>
@@ -1079,7 +1082,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:M18"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="12.1111111111111" style="2" customWidth="1"/>
@@ -1091,11 +1094,11 @@
     <col min="8" max="8" width="10" style="3" customWidth="1"/>
     <col min="9" max="9" width="13" style="3" customWidth="1"/>
     <col min="10" max="10" width="6.33333333333333" style="2" customWidth="1"/>
-    <col min="11" max="11" width="10.7777777777778" style="3"/>
-    <col min="12" max="12" width="9" style="2"/>
+    <col min="11" max="12" width="10.7777777777778" style="3"/>
+    <col min="13" max="13" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="28.8" spans="1:12">
+    <row r="1" s="1" customFormat="1" ht="43.2" spans="1:13">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1129,14 +1132,17 @@
       <c r="K1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="5"/>
-    </row>
-    <row r="2" spans="1:12">
+      <c r="L1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="5"/>
+    </row>
+    <row r="2" spans="1:13">
       <c r="A2" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C2" s="2">
         <v>10</v>
@@ -1160,12 +1166,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:13">
       <c r="A3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>12</v>
       </c>
       <c r="C3" s="2">
         <v>8</v>
@@ -1192,15 +1198,18 @@
         <v>10</v>
       </c>
       <c r="K3" s="3">
+        <v>46127</v>
+      </c>
+      <c r="L3" s="3">
         <v>46207</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:13">
       <c r="A4" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4" s="2">
         <v>8</v>
@@ -1227,15 +1236,18 @@
         <v>5</v>
       </c>
       <c r="K4" s="3">
+        <v>46127</v>
+      </c>
+      <c r="L4" s="3">
         <v>46207</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:13">
       <c r="A5" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C5" s="2">
         <v>0</v>
@@ -1253,15 +1265,18 @@
         <v>10</v>
       </c>
       <c r="K5" s="3">
+        <v>46127</v>
+      </c>
+      <c r="L5" s="3">
         <v>46207</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:13">
       <c r="A6" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C6" s="2">
         <v>1</v>
@@ -1279,15 +1294,18 @@
         <v>10</v>
       </c>
       <c r="K6" s="3">
+        <v>46127</v>
+      </c>
+      <c r="L6" s="3">
         <v>46207</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="1:13">
       <c r="A7" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C7" s="2">
         <v>1</v>
@@ -1305,12 +1323,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:12">
+    <row r="8" spans="1:13">
       <c r="A8" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C8" s="2">
         <v>0</v>
@@ -1337,15 +1355,18 @@
         <v>2</v>
       </c>
       <c r="K8" s="3">
+        <v>46127</v>
+      </c>
+      <c r="L8" s="3">
         <v>46207</v>
       </c>
     </row>
-    <row r="9" spans="1:12">
+    <row r="9" spans="1:13">
       <c r="A9" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C9" s="2">
         <v>0</v>
@@ -1363,15 +1384,18 @@
         <v>4</v>
       </c>
       <c r="K9" s="3">
+        <v>46127</v>
+      </c>
+      <c r="L9" s="3">
         <v>46207</v>
       </c>
     </row>
-    <row r="10" spans="1:12">
+    <row r="10" spans="1:13">
       <c r="A10" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C10" s="2">
         <v>2</v>
@@ -1395,12 +1419,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:12">
+    <row r="11" spans="1:13">
       <c r="A11" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C11" s="2">
         <v>0</v>
@@ -1415,15 +1439,18 @@
         <v>2</v>
       </c>
       <c r="K11" s="3">
+        <v>46127</v>
+      </c>
+      <c r="L11" s="3">
         <v>46207</v>
       </c>
     </row>
-    <row r="12" spans="1:12">
+    <row r="12" spans="1:13">
       <c r="A12" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C12" s="2">
         <v>1</v>
@@ -1438,12 +1465,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:12">
+    <row r="13" spans="1:13">
       <c r="A13" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C13" s="2">
         <v>7</v>
@@ -1458,12 +1485,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:12">
+    <row r="14" spans="1:13">
       <c r="A14" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>24</v>
       </c>
       <c r="C14" s="2">
         <v>1</v>
@@ -1478,12 +1505,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:12">
+    <row r="15" spans="1:13">
       <c r="A15" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C15" s="2">
         <v>1</v>
@@ -1498,12 +1525,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:12">
+    <row r="16" spans="1:13">
       <c r="A16" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C16" s="2">
         <v>3</v>
@@ -1520,10 +1547,10 @@
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C17" s="2">
         <v>3</v>
@@ -1540,10 +1567,10 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C18" s="2">
         <v>1</v>

</xml_diff>

<commit_message>
New Update on Serial number
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -29,11 +29,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="49">
   <si>
     <t>Model</t>
   </si>
   <si>
+    <t>Material Number</t>
+  </si>
+  <si>
     <t>Product Group</t>
   </si>
   <si>
@@ -70,58 +73,109 @@
     <t>LS0507EM</t>
   </si>
   <si>
+    <t>55F01390012B000</t>
+  </si>
+  <si>
     <t>Scissors</t>
   </si>
   <si>
     <t>LS0608E</t>
   </si>
   <si>
+    <t>55F02060007B000</t>
+  </si>
+  <si>
     <t>LS0808E</t>
   </si>
   <si>
+    <t>55F01480015B000</t>
+  </si>
+  <si>
     <t>LS0812E</t>
   </si>
   <si>
+    <t>55F01540011B000</t>
+  </si>
+  <si>
     <t>LS1012E</t>
   </si>
   <si>
+    <t>55F01500013B000</t>
+  </si>
+  <si>
     <t>LS1212E</t>
   </si>
   <si>
+    <t>55F01470012B000</t>
+  </si>
+  <si>
     <t>LS1412E</t>
   </si>
   <si>
+    <t>55F01850002B000</t>
+  </si>
+  <si>
     <t>LS1414E</t>
   </si>
   <si>
+    <t>55F02470006B000</t>
+  </si>
+  <si>
     <t>LS0610EC</t>
   </si>
   <si>
+    <t>55F02460008B000</t>
+  </si>
+  <si>
     <t>LS1216HC</t>
   </si>
   <si>
+    <t>55F01800003B000</t>
+  </si>
+  <si>
     <t>LS1623ERT</t>
   </si>
   <si>
+    <t>55F01700004B000</t>
+  </si>
+  <si>
     <t>LM09JE</t>
   </si>
   <si>
+    <t>55F02590012B000</t>
+  </si>
+  <si>
     <t>Boom</t>
   </si>
   <si>
     <t>LA14JE</t>
   </si>
   <si>
+    <t>55F01680006B000</t>
+  </si>
+  <si>
     <t>LA16JE</t>
   </si>
   <si>
+    <t>55F02140003B000</t>
+  </si>
+  <si>
     <t>LA20JE</t>
   </si>
   <si>
+    <t>55F01520002B000</t>
+  </si>
+  <si>
     <t>LT20JE</t>
   </si>
   <si>
+    <t>55F01120002B000</t>
+  </si>
+  <si>
     <t>LT26JE</t>
+  </si>
+  <si>
+    <t>55F01350002B000</t>
   </si>
 </sst>
 </file>
@@ -752,7 +806,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -768,8 +822,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1082,515 +1142,572 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="12.1111111111111" style="2" customWidth="1"/>
-    <col min="2" max="2" width="8.55555555555556" style="2" customWidth="1"/>
-    <col min="3" max="4" width="6.33333333333333" style="2" customWidth="1"/>
-    <col min="5" max="5" width="10.7777777777778" style="3"/>
-    <col min="6" max="6" width="9" style="2"/>
-    <col min="7" max="7" width="16.3333333333333" style="3" customWidth="1"/>
-    <col min="8" max="8" width="10" style="3" customWidth="1"/>
-    <col min="9" max="9" width="13" style="3" customWidth="1"/>
-    <col min="10" max="10" width="6.33333333333333" style="2" customWidth="1"/>
-    <col min="11" max="12" width="10.7777777777778" style="3"/>
-    <col min="13" max="13" width="9" style="2"/>
+    <col min="1" max="1" width="15.3518518518519" style="2" customWidth="1"/>
+    <col min="2" max="2" width="20.5833333333333" style="2" customWidth="1"/>
+    <col min="3" max="3" width="8.55555555555556" style="2" customWidth="1"/>
+    <col min="4" max="5" width="6.33333333333333" style="2" customWidth="1"/>
+    <col min="6" max="6" width="10.7777777777778" style="3"/>
+    <col min="7" max="7" width="9" style="2"/>
+    <col min="8" max="8" width="16.3333333333333" style="3" customWidth="1"/>
+    <col min="9" max="9" width="10" style="3" customWidth="1"/>
+    <col min="10" max="10" width="13" style="3" customWidth="1"/>
+    <col min="11" max="11" width="8.21296296296296" style="2" customWidth="1"/>
+    <col min="12" max="13" width="10.7777777777778" style="3"/>
+    <col min="14" max="14" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="43.2" spans="1:13">
+    <row r="1" s="1" customFormat="1" ht="43.2" spans="1:14">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="5"/>
+      <c r="M1" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="6"/>
     </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="2" t="s">
+    <row r="2" ht="28.8" spans="1:14">
+      <c r="A2" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="2">
+        <v>6</v>
+      </c>
+      <c r="E2" s="2">
+        <v>0</v>
+      </c>
+      <c r="G2" s="2">
+        <v>19</v>
+      </c>
+      <c r="H2" s="3">
+        <v>46092</v>
+      </c>
+      <c r="I2" s="3">
+        <v>46143</v>
+      </c>
+      <c r="J2" s="3">
+        <f>I2+45</f>
+        <v>46188</v>
+      </c>
+      <c r="K2" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" ht="28.8" spans="1:14">
+      <c r="A3" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="2">
+        <v>4</v>
+      </c>
+      <c r="E3" s="2">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2">
         <v>12</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="H3" s="3">
+        <v>46092</v>
+      </c>
+      <c r="I3" s="3">
+        <v>46143</v>
+      </c>
+      <c r="J3" s="3">
+        <f t="shared" ref="J3:J8" si="0">I3+45</f>
+        <v>46188</v>
+      </c>
+      <c r="K3" s="2">
+        <v>10</v>
+      </c>
+      <c r="L3" s="3">
+        <v>46134</v>
+      </c>
+      <c r="M3" s="3">
+        <f t="shared" ref="M3:M7" si="1">L3+45+35</f>
+        <v>46214</v>
+      </c>
+    </row>
+    <row r="4" ht="28.8" spans="1:14">
+      <c r="A4" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="2">
         <v>13</v>
       </c>
-      <c r="C2" s="2">
-        <v>6</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0</v>
-      </c>
-      <c r="F2" s="2">
-        <v>19</v>
-      </c>
-      <c r="G2" s="3">
+      <c r="E4" s="2">
+        <v>0</v>
+      </c>
+      <c r="G4" s="2">
+        <v>8</v>
+      </c>
+      <c r="H4" s="3">
         <v>46092</v>
       </c>
-      <c r="H2" s="3">
+      <c r="I4" s="3">
         <v>46143</v>
       </c>
-      <c r="I2" s="3">
-        <f>H2+45</f>
-        <v>46188</v>
-      </c>
-      <c r="J2" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="2">
-        <v>4</v>
-      </c>
-      <c r="D3" s="2">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3"/>
-      <c r="F3" s="2">
-        <v>12</v>
-      </c>
-      <c r="G3" s="3">
-        <v>46092</v>
-      </c>
-      <c r="H3" s="3">
-        <v>46143</v>
-      </c>
-      <c r="I3" s="3">
-        <f t="shared" ref="I3:I8" si="0">H3+45</f>
-        <v>46188</v>
-      </c>
-      <c r="J3" s="2">
-        <v>10</v>
-      </c>
-      <c r="K3" s="3">
-        <v>46134</v>
-      </c>
-      <c r="L3" s="3">
-        <f t="shared" ref="L3:L6" si="1">K3+45+35</f>
-        <v>46214</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="2">
-        <v>13</v>
-      </c>
-      <c r="D4" s="2">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3"/>
-      <c r="F4" s="2">
-        <v>8</v>
-      </c>
-      <c r="G4" s="3">
-        <v>46092</v>
-      </c>
-      <c r="H4" s="3">
-        <v>46143</v>
-      </c>
-      <c r="I4" s="3">
+      <c r="J4" s="3">
         <f t="shared" si="0"/>
         <v>46188</v>
       </c>
-      <c r="J4" s="2">
+      <c r="K4" s="2">
         <v>5</v>
       </c>
-      <c r="K4" s="3">
+      <c r="L4" s="3">
         <v>46134</v>
       </c>
-      <c r="L4" s="3">
+      <c r="M4" s="3">
         <f t="shared" si="1"/>
         <v>46214</v>
       </c>
     </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="2">
+    <row r="5" ht="28.8" spans="1:14">
+      <c r="A5" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="2">
         <v>18</v>
       </c>
-      <c r="D5" s="2">
-        <v>0</v>
-      </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="2">
-        <v>0</v>
-      </c>
-      <c r="J5" s="2">
+      <c r="E5" s="2">
+        <v>0</v>
+      </c>
+      <c r="G5" s="2">
+        <v>0</v>
+      </c>
+      <c r="K5" s="2">
         <v>10</v>
       </c>
-      <c r="K5" s="3">
+      <c r="L5" s="3">
         <v>46134</v>
       </c>
-      <c r="L5" s="3">
+      <c r="M5" s="3">
         <f t="shared" si="1"/>
         <v>46214</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="2">
+    <row r="6" ht="28.8" spans="1:14">
+      <c r="A6" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="2">
         <v>5</v>
       </c>
-      <c r="D6" s="2">
-        <v>0</v>
-      </c>
-      <c r="E6" s="3"/>
-      <c r="F6" s="2">
-        <v>0</v>
-      </c>
-      <c r="J6" s="2">
+      <c r="E6" s="2">
+        <v>0</v>
+      </c>
+      <c r="G6" s="2">
+        <v>0</v>
+      </c>
+      <c r="K6" s="2">
         <v>10</v>
       </c>
-      <c r="K6" s="3">
+      <c r="L6" s="3">
         <v>46134</v>
       </c>
-      <c r="L6" s="3">
+      <c r="M6" s="3">
         <f t="shared" si="1"/>
         <v>46214</v>
       </c>
     </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="2">
-        <v>0</v>
+    <row r="7" ht="28.8" spans="1:14">
+      <c r="A7" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="D7" s="2">
         <v>0</v>
       </c>
-      <c r="E7" s="3"/>
-      <c r="F7" s="2">
-        <v>0</v>
-      </c>
-      <c r="J7" s="2">
-        <v>0</v>
+      <c r="E7" s="2">
+        <v>0</v>
+      </c>
+      <c r="G7" s="2">
+        <v>0</v>
+      </c>
+      <c r="K7" s="2">
+        <v>3</v>
+      </c>
+      <c r="L7" s="3">
+        <v>46134</v>
+      </c>
+      <c r="M7" s="3">
+        <f t="shared" si="1"/>
+        <v>46214</v>
       </c>
     </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" s="2">
-        <v>0</v>
+    <row r="8" ht="28.8" spans="1:14">
+      <c r="A8" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="D8" s="2">
+        <v>0</v>
+      </c>
+      <c r="E8" s="2">
         <v>2</v>
       </c>
-      <c r="E8" s="3">
+      <c r="F8" s="3">
         <v>46158</v>
       </c>
-      <c r="F8" s="2">
+      <c r="G8" s="2">
         <v>2</v>
       </c>
-      <c r="G8" s="3">
+      <c r="H8" s="3">
         <v>46092</v>
       </c>
-      <c r="H8" s="3">
+      <c r="I8" s="3">
         <v>46143</v>
       </c>
-      <c r="I8" s="3">
+      <c r="J8" s="3">
         <f t="shared" si="0"/>
         <v>46188</v>
       </c>
-      <c r="J8" s="2">
+      <c r="K8" s="2">
         <v>2</v>
       </c>
-      <c r="K8" s="3">
+      <c r="L8" s="3">
         <v>46134</v>
       </c>
-      <c r="L8" s="3">
-        <f t="shared" ref="L8:L11" si="2">K8+45+35</f>
+      <c r="M8" s="3">
+        <f t="shared" ref="M8:M11" si="2">L8+45+35</f>
         <v>46214</v>
       </c>
     </row>
-    <row r="9" spans="1:13">
-      <c r="A9" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="2">
-        <v>0</v>
+    <row r="9" ht="28.8" spans="1:14">
+      <c r="A9" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="D9" s="2">
+        <v>0</v>
+      </c>
+      <c r="E9" s="2">
         <v>2</v>
       </c>
-      <c r="E9" s="3">
+      <c r="F9" s="3">
         <v>46158</v>
       </c>
-      <c r="F9" s="2">
-        <v>0</v>
-      </c>
-      <c r="J9" s="2">
+      <c r="G9" s="2">
+        <v>0</v>
+      </c>
+      <c r="K9" s="2">
         <v>4</v>
       </c>
-      <c r="K9" s="3">
+      <c r="L9" s="3">
         <v>46134</v>
       </c>
-      <c r="L9" s="3">
+      <c r="M9" s="3">
         <f t="shared" si="2"/>
         <v>46214</v>
       </c>
     </row>
-    <row r="10" spans="1:13">
-      <c r="A10" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B10" s="2" t="s">
+    <row r="10" ht="28.8" spans="1:14">
+      <c r="A10" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" s="2">
+        <v>2</v>
+      </c>
+      <c r="E10" s="2">
+        <v>0</v>
+      </c>
+      <c r="G10" s="2">
+        <v>10</v>
+      </c>
+      <c r="H10" s="3">
+        <v>46092</v>
+      </c>
+      <c r="I10" s="3">
+        <v>46143</v>
+      </c>
+      <c r="J10" s="3">
+        <f>I10+45</f>
+        <v>46188</v>
+      </c>
+      <c r="K10" s="2">
         <v>13</v>
       </c>
-      <c r="C10" s="2">
-        <v>2</v>
-      </c>
-      <c r="D10" s="2">
-        <v>0</v>
-      </c>
-      <c r="F10" s="2">
-        <v>10</v>
-      </c>
-      <c r="G10" s="3">
-        <v>46092</v>
-      </c>
-      <c r="H10" s="3">
-        <v>46143</v>
-      </c>
-      <c r="I10" s="3">
-        <f>H10+45</f>
-        <v>46188</v>
-      </c>
-      <c r="J10" s="2">
-        <v>13</v>
-      </c>
-      <c r="K10" s="3">
+      <c r="L10" s="3">
         <v>46141</v>
       </c>
-      <c r="L10" s="3">
+      <c r="M10" s="3">
         <f t="shared" si="2"/>
         <v>46221</v>
       </c>
     </row>
-    <row r="11" spans="1:13">
-      <c r="A11" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C11" s="2">
-        <v>0</v>
+    <row r="11" ht="28.8" spans="1:14">
+      <c r="A11" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="D11" s="2">
         <v>0</v>
       </c>
-      <c r="F11" s="2">
-        <v>0</v>
-      </c>
-      <c r="J11" s="2">
+      <c r="E11" s="2">
+        <v>0</v>
+      </c>
+      <c r="G11" s="2">
+        <v>0</v>
+      </c>
+      <c r="K11" s="2">
         <v>2</v>
       </c>
-      <c r="K11" s="3">
+      <c r="L11" s="3">
         <v>46134</v>
       </c>
-      <c r="L11" s="3">
+      <c r="M11" s="3">
         <f t="shared" si="2"/>
         <v>46214</v>
       </c>
     </row>
-    <row r="12" spans="1:13">
-      <c r="A12" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C12" s="2">
+    <row r="12" ht="28.8" spans="1:14">
+      <c r="A12" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" s="2">
         <v>1</v>
       </c>
-      <c r="D12" s="2">
-        <v>0</v>
-      </c>
-      <c r="F12" s="2">
-        <v>0</v>
-      </c>
-      <c r="J12" s="2">
+      <c r="E12" s="2">
+        <v>0</v>
+      </c>
+      <c r="G12" s="2">
+        <v>0</v>
+      </c>
+      <c r="K12" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:13">
-      <c r="A13" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C13" s="2">
+    <row r="13" ht="28.8" spans="1:14">
+      <c r="A13" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" s="2">
         <v>7</v>
       </c>
-      <c r="D13" s="2">
-        <v>0</v>
-      </c>
-      <c r="F13" s="2">
+      <c r="E13" s="2">
+        <v>0</v>
+      </c>
+      <c r="G13" s="2">
         <v>8</v>
       </c>
-      <c r="J13" s="2">
+      <c r="K13" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:13">
-      <c r="A14" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C14" s="2">
+    <row r="14" ht="28.8" spans="1:14">
+      <c r="A14" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D14" s="2">
         <v>1</v>
       </c>
-      <c r="D14" s="2">
-        <v>0</v>
-      </c>
-      <c r="F14" s="2">
-        <v>0</v>
-      </c>
-      <c r="J14" s="2">
+      <c r="E14" s="2">
+        <v>0</v>
+      </c>
+      <c r="G14" s="2">
+        <v>0</v>
+      </c>
+      <c r="K14" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:13">
-      <c r="A15" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C15" s="2">
+    <row r="15" ht="28.8" spans="1:14">
+      <c r="A15" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D15" s="2">
         <v>1</v>
       </c>
-      <c r="D15" s="2">
-        <v>0</v>
-      </c>
-      <c r="F15" s="2">
-        <v>0</v>
-      </c>
-      <c r="J15" s="2">
+      <c r="E15" s="2">
+        <v>0</v>
+      </c>
+      <c r="G15" s="2">
+        <v>0</v>
+      </c>
+      <c r="K15" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:13">
-      <c r="A16" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C16" s="2">
+    <row r="16" ht="28.8" spans="1:14">
+      <c r="A16" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D16" s="2">
         <v>3</v>
       </c>
-      <c r="D16" s="2">
-        <v>0</v>
-      </c>
-      <c r="F16" s="2">
-        <v>0</v>
-      </c>
-      <c r="J16" s="2">
+      <c r="E16" s="2">
+        <v>0</v>
+      </c>
+      <c r="G16" s="2">
+        <v>0</v>
+      </c>
+      <c r="K16" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:10">
-      <c r="A17" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C17" s="2">
+    <row r="17" ht="28.8" spans="1:11">
+      <c r="A17" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" s="2">
         <v>3</v>
       </c>
-      <c r="D17" s="2">
-        <v>0</v>
-      </c>
-      <c r="F17" s="2">
-        <v>0</v>
-      </c>
-      <c r="J17" s="2">
+      <c r="E17" s="2">
+        <v>0</v>
+      </c>
+      <c r="G17" s="2">
+        <v>0</v>
+      </c>
+      <c r="K17" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:10">
-      <c r="A18" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C18" s="2">
+    <row r="18" ht="28.8" spans="1:11">
+      <c r="A18" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D18" s="2">
         <v>1</v>
       </c>
-      <c r="D18" s="2">
-        <v>0</v>
-      </c>
-      <c r="F18" s="2">
-        <v>0</v>
-      </c>
-      <c r="J18" s="2">
+      <c r="E18" s="2">
+        <v>0</v>
+      </c>
+      <c r="G18" s="2">
+        <v>0</v>
+      </c>
+      <c r="K18" s="2">
         <v>0</v>
       </c>
     </row>

</xml_diff>